<commit_message>
Fix 01_Auditing_Formulas.xlsx: correct column refs and remove invalid formula characters
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-08/01_Auditing_Formulas.xlsx
+++ b/rFLA300/chapter-08/01_Auditing_Formulas.xlsx
@@ -146,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -211,7 +211,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -224,11 +223,17 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -599,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C28"/>
+  <dimension ref="B2:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -610,14 +615,14 @@
     <row r="2" ht="36" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Chapter 8 · Auditing Formulas</t>
+          <t>Chapter 8 - Auditing Formulas</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Student Practice Workbook · rFLA300 Data Analytics with Excel</t>
+          <t>Student Practice Workbook - rFLA300 Data Analytics with Excel</t>
         </is>
       </c>
     </row>
@@ -628,250 +633,230 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>This workbook covers formula auditing tools in Excel. You will practice tracing which cells a formula uses (precedents) and which cells depend on it (dependents), evaluate formulas step by step, find and fix circular references, and use the Watch Window to monitor key cells.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
+          <t>This workbook covers formula auditing tools in Excel. You will practice tracing which cells a formula uses (precedents) and which cells depend on it (dependents).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Auditing tools help you understand how formulas work and catch errors before they affect your results.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
+          <t>You will also evaluate formulas step by step, find and fix circular references, and use the Watch Window to monitor key cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Complete the sheets in order. Each sheet builds on the previous one.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="5" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Sheet Guide</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Sales_Data</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Sample sales dataset used throughout all lessons</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="B11" s="8" t="inlineStr">
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Precedents_Dependents</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Trace which cells feed into a formula and which cells use it</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Evaluate_Formulas</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Step through formulas one calculation at a time</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="8" t="inlineStr">
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Circular_Reference</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Find and fix circular reference errors</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="6" t="inlineStr">
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Watch_Window</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Monitor key cells without scrolling</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="10" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Key Terms</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="6" t="inlineStr">
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Precedents</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Cells that a formula refers to (the formula uses these cells)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="8" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Dependents</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>Cells that contain formulas that refer to the selected cell</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="6" t="inlineStr">
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Evaluate Formula</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Tool that calculates a formula one step at a time</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="8" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Circular Reference</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>A formula that refers to its own cell, directly or indirectly</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="6" t="inlineStr">
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Watch Window</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>A panel that shows the value of selected cells at all times</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="8" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Tracer Arrow</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Blue arrow drawn by Excel to show precedent or dependent links</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="11" t="inlineStr">
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>How to Use This Workbook</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Step 1</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Start on the Sales_Data sheet to understand the dataset.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Move to Precedents_Dependents and follow the step-by-step instructions.</t>
-        </is>
-      </c>
-    </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Step 3</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Open the Formulas tab in Excel to find the Formula Auditing group.</t>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Step 1: Start on the Sales_Data sheet to understand the dataset.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Step 4</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Complete each sheet before moving to the next.</t>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Step 2: Move to Precedents_Dependents and follow the step-by-step instructions.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Step 5</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Use the Watch Window sheet last — it pulls values from all other sheets.</t>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Step 3: Open the Formulas tab in Excel to find the Formula Auditing group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Step 4: Complete each sheet before moving to the next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Step 5: Use the Watch Window sheet last - it monitors values from all other sheets.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="14">
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B27:C27"/>
     <mergeCell ref="B8:C8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -888,28 +873,29 @@
   <dimension ref="B2:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>Sales Data · Chapter 8 Lesson Dataset</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>Sales Data - Chapter 8 Lesson Dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>This dataset is used across all Chapter 8 lessons. Do not edit values in columns B–G. Use columns H and I for your formula work.</t>
+          <t>This dataset is used across all Chapter 8 lessons. Columns H-J contain formulas to practice auditing.</t>
         </is>
       </c>
     </row>
@@ -931,7 +917,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Units Sold</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
@@ -941,7 +927,7 @@
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>Discount %</t>
+          <t>Disc %</t>
         </is>
       </c>
       <c r="H5" s="14" t="inlineStr">
@@ -951,12 +937,12 @@
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
-          <t>Commission (10%)</t>
+          <t>Commission</t>
         </is>
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>Bonus Eligible?</t>
+          <t>Bonus?</t>
         </is>
       </c>
     </row>
@@ -983,16 +969,16 @@
       <c r="G6" s="17" t="n">
         <v>0.05</v>
       </c>
-      <c r="H6" s="15">
-        <f>D6*E6*(1-F6)</f>
-        <v/>
-      </c>
-      <c r="I6" s="15">
-        <f>G6*0.10</f>
+      <c r="H6" s="16">
+        <f>E6*F6*(1-G6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="16">
+        <f>H6*0.10</f>
         <v/>
       </c>
       <c r="J6" s="15">
-        <f>IF(D6&gt;=100,"Yes","No")</f>
+        <f>IF(E6&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1019,16 +1005,16 @@
       <c r="G7" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="H7" s="18">
-        <f>D7*E7*(1-F7)</f>
-        <v/>
-      </c>
-      <c r="I7" s="18">
-        <f>G7*0.10</f>
+      <c r="H7" s="19">
+        <f>E7*F7*(1-G7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="19">
+        <f>H7*0.10</f>
         <v/>
       </c>
       <c r="J7" s="18">
-        <f>IF(D7&gt;=100,"Yes","No")</f>
+        <f>IF(E7&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1055,16 +1041,16 @@
       <c r="G8" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="15">
-        <f>D8*E8*(1-F8)</f>
-        <v/>
-      </c>
-      <c r="I8" s="15">
-        <f>G8*0.10</f>
+      <c r="H8" s="16">
+        <f>E8*F8*(1-G8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="16">
+        <f>H8*0.10</f>
         <v/>
       </c>
       <c r="J8" s="15">
-        <f>IF(D8&gt;=100,"Yes","No")</f>
+        <f>IF(E8&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1091,16 +1077,16 @@
       <c r="G9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="H9" s="18">
-        <f>D9*E9*(1-F9)</f>
-        <v/>
-      </c>
-      <c r="I9" s="18">
-        <f>G9*0.10</f>
+      <c r="H9" s="19">
+        <f>E9*F9*(1-G9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="19">
+        <f>H9*0.10</f>
         <v/>
       </c>
       <c r="J9" s="18">
-        <f>IF(D9&gt;=100,"Yes","No")</f>
+        <f>IF(E9&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1127,16 +1113,16 @@
       <c r="G10" s="17" t="n">
         <v>0.05</v>
       </c>
-      <c r="H10" s="15">
-        <f>D10*E10*(1-F10)</f>
-        <v/>
-      </c>
-      <c r="I10" s="15">
-        <f>G10*0.10</f>
+      <c r="H10" s="16">
+        <f>E10*F10*(1-G10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="16">
+        <f>H10*0.10</f>
         <v/>
       </c>
       <c r="J10" s="15">
-        <f>IF(D10&gt;=100,"Yes","No")</f>
+        <f>IF(E10&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1163,16 +1149,16 @@
       <c r="G11" s="20" t="n">
         <v>0.2</v>
       </c>
-      <c r="H11" s="18">
-        <f>D11*E11*(1-F11)</f>
-        <v/>
-      </c>
-      <c r="I11" s="18">
-        <f>G11*0.10</f>
+      <c r="H11" s="19">
+        <f>E11*F11*(1-G11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="19">
+        <f>H11*0.10</f>
         <v/>
       </c>
       <c r="J11" s="18">
-        <f>IF(D11&gt;=100,"Yes","No")</f>
+        <f>IF(E11&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1199,16 +1185,16 @@
       <c r="G12" s="17" t="n">
         <v>0.1</v>
       </c>
-      <c r="H12" s="15">
-        <f>D12*E12*(1-F12)</f>
-        <v/>
-      </c>
-      <c r="I12" s="15">
-        <f>G12*0.10</f>
+      <c r="H12" s="16">
+        <f>E12*F12*(1-G12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="16">
+        <f>H12*0.10</f>
         <v/>
       </c>
       <c r="J12" s="15">
-        <f>IF(D12&gt;=100,"Yes","No")</f>
+        <f>IF(E12&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1235,16 +1221,16 @@
       <c r="G13" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="18">
-        <f>D13*E13*(1-F13)</f>
-        <v/>
-      </c>
-      <c r="I13" s="18">
-        <f>G13*0.10</f>
+      <c r="H13" s="19">
+        <f>E13*F13*(1-G13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="19">
+        <f>H13*0.10</f>
         <v/>
       </c>
       <c r="J13" s="18">
-        <f>IF(D13&gt;=100,"Yes","No")</f>
+        <f>IF(E13&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1271,16 +1257,16 @@
       <c r="G14" s="17" t="n">
         <v>0.05</v>
       </c>
-      <c r="H14" s="15">
-        <f>D14*E14*(1-F14)</f>
-        <v/>
-      </c>
-      <c r="I14" s="15">
-        <f>G14*0.10</f>
+      <c r="H14" s="16">
+        <f>E14*F14*(1-G14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="16">
+        <f>H14*0.10</f>
         <v/>
       </c>
       <c r="J14" s="15">
-        <f>IF(D14&gt;=100,"Yes","No")</f>
+        <f>IF(E14&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1307,16 +1293,16 @@
       <c r="G15" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="H15" s="18">
-        <f>D15*E15*(1-F15)</f>
-        <v/>
-      </c>
-      <c r="I15" s="18">
-        <f>G15*0.10</f>
+      <c r="H15" s="19">
+        <f>E15*F15*(1-G15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="19">
+        <f>H15*0.10</f>
         <v/>
       </c>
       <c r="J15" s="18">
-        <f>IF(D15&gt;=100,"Yes","No")</f>
+        <f>IF(E15&gt;=100,"Yes","No")</f>
         <v/>
       </c>
     </row>
@@ -1326,39 +1312,39 @@
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="C16" s="22" t="n"/>
-      <c r="D16" s="22" t="n"/>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
       <c r="E16" s="21">
-        <f>SUM(D6:D15)</f>
+        <f>SUM(E6:E15)</f>
         <v/>
       </c>
       <c r="F16" s="21">
-        <f>AVERAGE(E6:E15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="22" t="n"/>
+        <f>AVERAGE(F6:F15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="21" t="n"/>
       <c r="H16" s="21">
-        <f>SUM(G6:G15)</f>
+        <f>SUM(H6:H15)</f>
         <v/>
       </c>
       <c r="I16" s="21">
-        <f>SUM(H6:H15)</f>
-        <v/>
-      </c>
-      <c r="J16" s="22" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="23" t="inlineStr">
-        <is>
-          <t>Lesson Tip: Click any cell in column H or I and go to Formulas tab → Trace Precedents to see which cells that formula uses.</t>
+        <f>SUM(I6:I15)</f>
+        <v/>
+      </c>
+      <c r="J16" s="21" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Tip: Click cell H6 and go to Formulas tab &gt; Trace Precedents to see which cells that formula uses.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B18:I18"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1371,10 +1357,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G27"/>
+  <dimension ref="B2:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -1386,21 +1372,21 @@
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>Lesson 1 · Trace Precedents and Dependents</t>
+          <t>Lesson 1 - Trace Precedents and Dependents</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Objective: Use Excel's Trace Precedents and Trace Dependents buttons to visualize how formulas connect to data cells.</t>
+          <t>Objective: Use Trace Precedents and Trace Dependents to visualize how formulas connect to data cells.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>What Are Precedents and Dependents?</t>
+          <t>Precedents and Dependents Explained</t>
         </is>
       </c>
     </row>
@@ -1410,9 +1396,9 @@
           <t>PRECEDENTS</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Cells that your formula USES. Think: 'What feeds this formula?'</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Cells that your formula USES. What feeds this formula?</t>
         </is>
       </c>
     </row>
@@ -1422,9 +1408,9 @@
           <t>DEPENDENTS</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>Cells that USE your cell. Think: 'What formula needs this value?'</t>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Cells that USE your cell. What formula needs this value?</t>
         </is>
       </c>
     </row>
@@ -1434,9 +1420,9 @@
           <t>Tracer Arrows</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Blue arrows drawn by Excel to show the connections visually.</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Blue arrows Excel draws to show the connections visually.</t>
         </is>
       </c>
     </row>
@@ -1446,16 +1432,16 @@
           <t>Remove Arrows</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Click Remove Arrows to clear all tracer arrows when done.</t>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Click Remove Arrows on the Formulas tab to clear all arrows.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Practice Dataset — Regional Sales Summary</t>
+          <t>Practice Dataset - Regional Sales Summary</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1495,7 @@
       <c r="F13" s="15" t="n">
         <v>15600</v>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="23">
         <f>SUM(C13:F13)</f>
         <v/>
       </c>
@@ -1532,7 +1518,7 @@
       <c r="F14" s="18" t="n">
         <v>12300</v>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="23">
         <f>SUM(C14:F14)</f>
         <v/>
       </c>
@@ -1555,7 +1541,7 @@
       <c r="F15" s="15" t="n">
         <v>16800</v>
       </c>
-      <c r="G15" s="24">
+      <c r="G15" s="23">
         <f>SUM(C15:F15)</f>
         <v/>
       </c>
@@ -1578,12 +1564,12 @@
       <c r="F16" s="18" t="n">
         <v>11200</v>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="23">
         <f>SUM(C16:F16)</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
+    <row r="17" ht="18" customHeight="1">
       <c r="B17" s="21" t="inlineStr">
         <is>
           <t>Grand Total</t>
@@ -1625,7 +1611,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Click on cell G13 (North Annual Total). This cell contains =SUM(C13:F13).</t>
+          <t>Click on cell G13 (North Annual Total). It contains =SUM(C13:F13).</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1623,7 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Go to the Formulas tab → Formula Auditing group → click Trace Precedents.</t>
+          <t>Go to Formulas tab &gt; Formula Auditing group &gt; click Trace Precedents.</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1647,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Now click cell C13 (Q1 North Sales). Click Trace Dependents.</t>
+          <t>Click cell C13 (Q1 North Sales). Click Trace Dependents.</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1659,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Arrows show G13 and C17 (Grand Total) both depend on C13.</t>
+          <t>Arrows show G13 and C17 (Grand Total Q1) both depend on C13.</t>
         </is>
       </c>
     </row>
@@ -1697,14 +1683,14 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Repeat with cells in row 14, 15, and 16 to see similar patterns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="36" customHeight="1">
-      <c r="B27" s="23" t="inlineStr">
-        <is>
-          <t>Self-Check: After tracing G17 (Grand Total), how many precedent arrows appear? Answer: 4 arrows — one from each regional Annual Total in G13:G16.</t>
+          <t>Repeat with cells in rows 14, 15, and 16 to see similar patterns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>Self-Check: After tracing G17 (Grand Total), how many precedent arrows appear? Answer: 4 arrows, one from each G13:G16.</t>
         </is>
       </c>
     </row>
@@ -1713,18 +1699,18 @@
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B19:G19"/>
+    <mergeCell ref="C7:G7"/>
     <mergeCell ref="C21:G21"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="C23:G23"/>
     <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C9:G9"/>
     <mergeCell ref="B11:G11"/>
     <mergeCell ref="C26:G26"/>
   </mergeCells>
@@ -1742,7 +1728,7 @@
   <dimension ref="B2:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -1753,7 +1739,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>Lesson 2 · Evaluate Formulas Step by Step</t>
+          <t>Lesson 2 - Evaluate Formulas Step by Step</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1767,7 @@
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>2. Go to the Formulas tab → Formula Auditing group.</t>
+          <t>2. Go to the Formulas tab &gt; Formula Auditing group.</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1795,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>6. Click Step In to enter a nested function, or Step Out to return to the outer formula.</t>
+          <t>6. Click Step In to enter a nested function, or Step Out to return.</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1809,7 @@
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Practice Formulas — Step Through Each One</t>
+          <t>Practice Formulas - Step Through Each One</t>
         </is>
       </c>
     </row>
@@ -1866,7 +1852,7 @@
       <c r="D16" s="15" t="n">
         <v>0.12</v>
       </c>
-      <c r="E16" s="24">
+      <c r="E16" s="23">
         <f>C16*D16</f>
         <v/>
       </c>
@@ -1888,7 +1874,7 @@
       <c r="D17" s="18" t="n">
         <v>0.08</v>
       </c>
-      <c r="E17" s="24">
+      <c r="E17" s="23">
         <f>C17*D17</f>
         <v/>
       </c>
@@ -1910,7 +1896,7 @@
       <c r="D18" s="15" t="n">
         <v>0.08</v>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="23">
         <f>C18*(1-D18)</f>
         <v/>
       </c>
@@ -1932,13 +1918,13 @@
       <c r="D19" s="18" t="n">
         <v>0.1</v>
       </c>
-      <c r="E19" s="24">
+      <c r="E19" s="23">
         <f>IF(C19&gt;5000,C19*D19,C19*0.05)</f>
         <v/>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>10% if revenue &gt; 5000, else 5%</t>
+          <t>10% if revenue over 5000, else 5%</t>
         </is>
       </c>
     </row>
@@ -1954,13 +1940,13 @@
       <c r="D20" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="23">
         <f>IF(C20&gt;=D20,"Pass","Fail")</f>
         <v/>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Pass if score &gt;= 70</t>
+          <t>Pass if score is 70 or above</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1962,7 @@
       <c r="D21" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E21" s="24">
+      <c r="E21" s="23">
         <f>ROUND(C21,D21)</f>
         <v/>
       </c>
@@ -1987,9 +1973,9 @@
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>Tip: Start with row 19 — the nested IF formula. Use Step In when Excel shows the IF function underlined to enter it and watch each condition evaluate.</t>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Tip: Start with row 19 (the Commission IF formula). Use Step In when the IF function is underlined to watch each condition evaluate.</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2008,17 @@
   <dimension ref="B2:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="25" t="inlineStr">
-        <is>
-          <t>Lesson 3 · Circular References — Find and Fix</t>
+      <c r="B2" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 3 - Circular References: Find and Fix</t>
         </is>
       </c>
     </row>
@@ -2053,9 +2039,9 @@
     <row r="6" ht="60" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>A circular reference occurs when a formula refers — directly or indirectly — to the cell that contains the formula itself.
-Example: If cell B10 contains =B10+1, Excel cannot calculate the answer because the answer depends on itself.
-Excel will show a warning message and the status bar may display 'Circular References'.</t>
+          <t>A circular reference occurs when a formula refers to the cell that contains the formula itself.
+Example: If cell B10 contains =B10+1, Excel cannot calculate because the answer depends on itself.
+Excel shows a warning and the status bar displays 'Circular References: [cell]'.</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2057,7 @@
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>1. Go to the Formulas tab → Formula Auditing group.</t>
+          <t>1. Go to the Formulas tab &gt; Formula Auditing group.</t>
         </is>
       </c>
     </row>
@@ -2085,42 +2071,42 @@
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>3. Click Circular References — Excel will show the cell addresses that have circular references.</t>
+          <t>3. Click Circular References - Excel lists the affected cell addresses.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>4. Click on a cell address in the list to navigate to that cell.</t>
+          <t>4. Click a cell address in the list to jump to that cell.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>5. Look at the formula and identify which part refers to the formula's own cell.</t>
+          <t>5. Look at the formula and find which part refers to the formula's own cell.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>6. Fix the formula by changing the cell reference to a different cell.</t>
+          <t>6. Fix the formula by changing the reference to a different cell.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="26" t="inlineStr">
-        <is>
-          <t>Practice: Find and Fix These Circular References</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>Practice: Identify the Problem in Each Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>The table below contains intentional errors. Identify the circular reference in each formula and write the corrected version in column E.</t>
+          <t>Read the description of each broken formula below. Write the corrected formula in column E.</t>
         </is>
       </c>
     </row>
@@ -2137,99 +2123,95 @@
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>Broken Formula (in column C)</t>
+          <t>Problem Formula (text)</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Corrected Formula — Type Here</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="25" customHeight="1">
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Total Sales</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
+          <t>Corrected Formula - Write Here</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Total Units Sold</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="D21" s="27" t="inlineStr">
-        <is>
-          <t>← =C21+D21</t>
-        </is>
+      <c r="D21" s="27">
+        <f>SUM(B21:B24) entered in B21 - range includes own cell</f>
+        <v/>
       </c>
       <c r="E21" s="28" t="inlineStr">
         <is>
-          <t>Fix: change to =C22+C23 or a valid range</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="25" customHeight="1">
-      <c r="B22" s="9" t="inlineStr">
+          <t>Fix: use SUM over only the data rows, exclude row 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="B22" s="29" t="inlineStr">
         <is>
           <t>Tax Amount</t>
         </is>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="27" t="inlineStr">
-        <is>
-          <t>← =C22*0.07</t>
-        </is>
+      <c r="D22" s="27">
+        <f>C22*0.07 but C22 is this cell - refers to itself</f>
+        <v/>
       </c>
       <c r="E22" s="28" t="inlineStr">
         <is>
-          <t>Fix: reference the correct sales cell, not this cell</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="25" customHeight="1">
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Net Revenue</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="n">
+          <t>Fix: reference the correct sales cell, e.g. =C21*0.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Running Total</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="27" t="inlineStr">
-        <is>
-          <t>← =C21-C23</t>
-        </is>
+      <c r="D23" s="27">
+        <f>D23+D22 where D23 is this cell</f>
+        <v/>
       </c>
       <c r="E23" s="28" t="inlineStr">
         <is>
-          <t>This formula depends on C21 which may also be broken</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="25" customHeight="1">
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Running Sum</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="n">
+          <t>Fix: =D22 + [the value above], not the current cell</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="C24" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="27" t="inlineStr">
-        <is>
-          <t>← =SUM(B21:B24)</t>
-        </is>
+      <c r="D24" s="27">
+        <f>SUM(E20:E24) entered in E24 - includes E24 itself</f>
+        <v/>
       </c>
       <c r="E24" s="28" t="inlineStr">
         <is>
-          <t>Fix: The range includes the formula cell itself</t>
+          <t>Fix: =SUM(E20:E23) - stop one row before the total cell</t>
         </is>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1">
-      <c r="B26" s="23" t="inlineStr">
-        <is>
-          <t>Remember: The status bar at the bottom of Excel shows 'Circular References: [cell]' when one exists. Always fix circular references — they return 0 or incorrect values.</t>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>Remember: The status bar at the bottom of Excel shows 'Circular References: [cell]' when one exists. Always fix circular references - they return 0 or wrong values.</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2246,7 @@
   <dimension ref="B2:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -2273,16 +2255,16 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="29" t="inlineStr">
-        <is>
-          <t>Lesson 4 · Use the Watch Window</t>
+      <c r="B2" s="30" t="inlineStr">
+        <is>
+          <t>Lesson 4 - Use the Watch Window</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Objective: Add key cells to the Watch Window so you can monitor their values while working elsewhere in the workbook.</t>
+          <t>Objective: Add key cells to the Watch Window to monitor their values while working elsewhere in the workbook.</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2298,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Formulas tab → Formula Auditing group → Watch Window</t>
+          <t>Formulas tab &gt; Formula Auditing group &gt; Watch Window</t>
         </is>
       </c>
     </row>
@@ -2340,14 +2322,14 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Click a cell or type the address; click Add</t>
+          <t>Click a cell or type the address, then click Add</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>4. The cell appears in the Watch list</t>
+          <t>4. Cell appears in the Watch list</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -2376,14 +2358,14 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Select it in the Watch Window list → click Delete Watch</t>
+          <t>Select it in the Watch Window list, then click Delete Watch</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Practice: Cells Worth Watching in This Workbook</t>
+          <t>Practice: Cells to Watch in This Workbook</t>
         </is>
       </c>
     </row>
@@ -2405,12 +2387,12 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Current Value</t>
+          <t>Formula to Expect</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Why Watch This?</t>
+          <t>Why Watch This</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2413,7 @@
         </is>
       </c>
       <c r="E19" s="7">
-        <f>SUM(G6:G15)</f>
+        <f>SUM(H6:H15)</f>
         <v/>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -2457,7 +2439,7 @@
         </is>
       </c>
       <c r="E20" s="9">
-        <f>SUM(H6:H15)</f>
+        <f>SUM(I6:I15)</f>
         <v/>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -2509,7 +2491,7 @@
         </is>
       </c>
       <c r="E22" s="9">
-        <f>IF(C19&gt;5000…)</f>
+        <f>IF(C19&gt;5000,...)</f>
         <v/>
       </c>
       <c r="F22" s="9" t="inlineStr">
@@ -2519,9 +2501,9 @@
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
-      <c r="B24" s="23" t="inlineStr">
-        <is>
-          <t>Practice: Add each cell above to your Watch Window, then navigate to the Circular_Reference sheet. Confirm that the Sales_Data totals still update in the Watch Window.</t>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>Practice: Add each cell above to your Watch Window, then navigate to the Circular_Reference sheet. Confirm the Sales_Data totals still update in the Watch Window.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: correct ARGB alpha channel from 00 to FF in all colors
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-08/01_Auditing_Formulas.xlsx
+++ b/rFLA300/chapter-08/01_Auditing_Formulas.xlsx
@@ -33,13 +33,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
@@ -54,7 +54,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
@@ -76,47 +76,47 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
+        <fgColor rgb="FF2E75B6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C55A11"/>
+        <fgColor rgb="FFC55A11"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00375623"/>
+        <fgColor rgb="FF375623"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
+        <fgColor rgb="FFC00000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -130,16 +130,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
     </border>
   </borders>
@@ -245,70 +245,70 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -600,7 +600,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F4E79"/>
+    <tabColor rgb="FF1F4E79"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -866,7 +866,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002E75B6"/>
+    <tabColor rgb="FF2E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1353,7 +1353,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002E75B6"/>
+    <tabColor rgb="FF2E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1721,7 +1721,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002E75B6"/>
+    <tabColor rgb="FF2E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2001,7 +2001,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00C55A11"/>
+    <tabColor rgb="FFC55A11"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2239,7 +2239,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00375623"/>
+    <tabColor rgb="FF375623"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>

<commit_message>
Fix: use write_string() to prevent = strings being parsed as formulas in sheet5
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-08/01_Auditing_Formulas.xlsx
+++ b/rFLA300/chapter-08/01_Auditing_Formulas.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="167">
   <si>
     <t>Chapter 8: Auditing Formulas</t>
   </si>
@@ -297,31 +297,19 @@
     <t>Go to Formulas tab &gt; Formula Auditing group &gt; Evaluate Formula.</t>
   </si>
   <si>
-    <t>The dialog shows: =E11*(1-D11). The underlined part is evaluated first.</t>
-  </si>
-  <si>
-    <t>Click "Evaluate" — E11 is replaced by its value (e.g. 63250).</t>
-  </si>
-  <si>
-    <t>Click "Evaluate" again — D11 is replaced by 0.22.</t>
+    <t>The dialog shows the formula. The underlined part is evaluated first.</t>
+  </si>
+  <si>
+    <t>Click "Evaluate" — the underlined reference is replaced by its value.</t>
+  </si>
+  <si>
+    <t>Click "Evaluate" repeatedly until the final result appears.</t>
   </si>
   <si>
     <t>Step 6:</t>
   </si>
   <si>
-    <t>Click "Evaluate" again — sees 63250*(1-0.22) = 63250*0.78.</t>
-  </si>
-  <si>
-    <t>Step 7:</t>
-  </si>
-  <si>
-    <t>Click "Evaluate" once more — final result appears.</t>
-  </si>
-  <si>
-    <t>Step 8:</t>
-  </si>
-  <si>
-    <t>Click "Close" when done.</t>
+    <t>Click "Restart" to start over, or "Close" when done.</t>
   </si>
   <si>
     <t>Circular References</t>
@@ -333,7 +321,7 @@
     <t>WHAT IS A CIRCULAR REFERENCE?</t>
   </si>
   <si>
-    <t>A circular reference occurs when a formula refers to its OWN cell, either directly or through a chain of references. Example: if A1 contains =A1+1, it refers to itself. Excel cannot calculate this and shows a warning. The status bar at the bottom of Excel displays "Circular References: A1".</t>
+    <t>A circular reference occurs when a formula refers to its OWN cell, either directly or through a chain of references. Excel cannot calculate this and shows a warning. The status bar at the bottom displays "Circular References: [cell]".</t>
   </si>
   <si>
     <t>HOW TO FIND THEM</t>
@@ -378,130 +366,157 @@
     <t>Or restructure the data so the calculation chain is linear (A feeds B, B feeds C — not C feeding back to A).</t>
   </si>
   <si>
-    <t>EXAMPLE (DO NOT COPY — for illustration only)</t>
+    <t>EXAMPLES (shown as text — do not use these as real formulas)</t>
   </si>
   <si>
     <t>Cell</t>
   </si>
   <si>
+    <t>Bad Formula (text)</t>
+  </si>
+  <si>
+    <t>Problem</t>
+  </si>
+  <si>
+    <t>Fix</t>
+  </si>
+  <si>
+    <t>B20</t>
+  </si>
+  <si>
+    <t>=B20+100</t>
+  </si>
+  <si>
+    <t>Directly references itself</t>
+  </si>
+  <si>
+    <t>=B19+100  (use the row above)</t>
+  </si>
+  <si>
+    <t>C20</t>
+  </si>
+  <si>
+    <t>=D20*1.1</t>
+  </si>
+  <si>
+    <t>D20 refers back to C20, creating a loop</t>
+  </si>
+  <si>
+    <t>Move calc to a separate helper column</t>
+  </si>
+  <si>
+    <t>D20</t>
+  </si>
+  <si>
+    <t>=SUM(D5:D20)</t>
+  </si>
+  <si>
+    <t>D20 is inside its own SUM range</t>
+  </si>
+  <si>
+    <t>=SUM(D5:D19)  (exclude current row)</t>
+  </si>
+  <si>
+    <t>Using the Watch Window</t>
+  </si>
+  <si>
+    <t>Formulas tab &gt; Formula Auditing &gt; Watch Window</t>
+  </si>
+  <si>
+    <t>WHAT IS THE WATCH WINDOW?</t>
+  </si>
+  <si>
+    <t>The Watch Window lets you monitor specific cells from ANY sheet without navigating there. It stays open as a floating panel and updates in real time. Useful for large workbooks where key results are on different sheets.</t>
+  </si>
+  <si>
+    <t>HOW TO ADD CELLS TO THE WATCH WINDOW</t>
+  </si>
+  <si>
+    <t>Open Watch Window</t>
+  </si>
+  <si>
+    <t>Formulas tab &gt; Formula Auditing group &gt; Watch Window</t>
+  </si>
+  <si>
+    <t>Add Watch</t>
+  </si>
+  <si>
+    <t>Click "Add Watch..." in the Watch Window toolbar</t>
+  </si>
+  <si>
+    <t>Select cell(s)</t>
+  </si>
+  <si>
+    <t>Select the cell(s) you want to monitor and click "Add"</t>
+  </si>
+  <si>
+    <t>View results</t>
+  </si>
+  <si>
+    <t>The Watch Window shows: Book, Sheet, Name, Cell, Value, Formula</t>
+  </si>
+  <si>
+    <t>Delete Watch</t>
+  </si>
+  <si>
+    <t>Select a watch entry and click "Delete Watch" to remove it</t>
+  </si>
+  <si>
+    <t>PRACTICE</t>
+  </si>
+  <si>
+    <t>Open the Watch Window (Formulas &gt; Watch Window).</t>
+  </si>
+  <si>
+    <t>Click "Add Watch" and select cells H3:H12 on the Sales_Data sheet.</t>
+  </si>
+  <si>
+    <t>Navigate to this Watch_Window sheet.</t>
+  </si>
+  <si>
+    <t>Change the price in Sales_Data cell F3 and watch H3 update in the Watch Window.</t>
+  </si>
+  <si>
+    <t>5.</t>
+  </si>
+  <si>
+    <t>Add the totals cell H13 (Total Net Revenue) to also monitor the grand total.</t>
+  </si>
+  <si>
+    <t>KEY FORMULAS IN SALES_DATA (for reference)</t>
+  </si>
+  <si>
     <t>Formula</t>
   </si>
   <si>
-    <t>Problem</t>
-  </si>
-  <si>
-    <t>Fix</t>
-  </si>
-  <si>
-    <t>B20</t>
-  </si>
-  <si>
-    <t>Directly references itself</t>
-  </si>
-  <si>
-    <t>C20</t>
-  </si>
-  <si>
-    <t>D20 contains =C20*2</t>
-  </si>
-  <si>
-    <t>Move calc to separate helper column</t>
-  </si>
-  <si>
-    <t>D20</t>
-  </si>
-  <si>
-    <t>D20 is inside its own SUM range</t>
-  </si>
-  <si>
-    <t>Using the Watch Window</t>
-  </si>
-  <si>
-    <t>Formulas tab &gt; Formula Auditing &gt; Watch Window</t>
-  </si>
-  <si>
-    <t>WHAT IS THE WATCH WINDOW?</t>
-  </si>
-  <si>
-    <t>The Watch Window lets you monitor specific cells from ANY sheet without having to navigate there. It stays open as a floating panel. When values change, the Watch Window updates in real time. Useful for large workbooks where key cells are on different sheets.</t>
-  </si>
-  <si>
-    <t>HOW TO ADD CELLS TO THE WATCH WINDOW</t>
-  </si>
-  <si>
-    <t>Open Watch Window</t>
-  </si>
-  <si>
-    <t>Formulas tab &gt; Formula Auditing group &gt; Watch Window</t>
-  </si>
-  <si>
-    <t>Add Watch</t>
-  </si>
-  <si>
-    <t>Click "Add Watch..." in the Watch Window toolbar</t>
-  </si>
-  <si>
-    <t>Select cell(s)</t>
-  </si>
-  <si>
-    <t>Select the cell(s) you want to monitor and click "Add"</t>
-  </si>
-  <si>
-    <t>View results</t>
-  </si>
-  <si>
-    <t>The Watch Window shows: Book, Sheet, Name, Cell, Value, Formula</t>
-  </si>
-  <si>
-    <t>Delete Watch</t>
-  </si>
-  <si>
-    <t>Select a watch entry and click "Delete Watch" to remove it</t>
-  </si>
-  <si>
-    <t>PRACTICE</t>
-  </si>
-  <si>
-    <t>Open the Watch Window (Formulas &gt; Watch Window).</t>
-  </si>
-  <si>
-    <t>Click "Add Watch" and select cells H3:H12 on the Sales_Data sheet.</t>
-  </si>
-  <si>
-    <t>Navigate to this Watch_Window sheet.</t>
-  </si>
-  <si>
-    <t>Change the price in Sales_Data F3 and watch H3 update in the Watch Window.</t>
-  </si>
-  <si>
-    <t>5.</t>
-  </si>
-  <si>
-    <t>Add the totals cell H13 (Total Net Revenue) to also monitor the grand total.</t>
-  </si>
-  <si>
-    <t>KEY FORMULA IN SALES_DATA (for reference)</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
-    <t>Value (example)</t>
+    <t>Note</t>
   </si>
   <si>
     <t>H3</t>
   </si>
   <si>
-    <t>Net Revenue = Units x Price x (1-Disc%)</t>
+    <t>=E3*F3*(1-G3)</t>
+  </si>
+  <si>
+    <t>Net Revenue = Units x Price x (1 minus Disc%)</t>
   </si>
   <si>
     <t>I3</t>
   </si>
   <si>
+    <t>=H3*0.10</t>
+  </si>
+  <si>
     <t>Commission = 10% of Net Revenue</t>
   </si>
   <si>
     <t>J3</t>
+  </si>
+  <si>
+    <t>=IF(E3&gt;=100,"Yes","No")</t>
   </si>
   <si>
     <t>Bonus eligibility based on units</t>
@@ -660,11 +675,15 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1743,7 +1762,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -1937,30 +1956,8 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
     </row>
-    <row r="20" spans="2:6">
-      <c r="B20" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="2:6">
-      <c r="B21" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="12">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
@@ -1973,8 +1970,6 @@
     <mergeCell ref="C17:F17"/>
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="C19:F19"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="C21:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1992,7 +1987,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="50" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2001,7 +1996,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2010,7 +2005,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="12" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -2019,7 +2014,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -2049,7 +2044,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="12" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -2058,37 +2053,37 @@
     </row>
     <row r="10" spans="1:5">
       <c r="B10" s="3" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5">
       <c r="B11" s="3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5">
       <c r="B12" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="12" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -2097,37 +2092,37 @@
     </row>
     <row r="14" spans="1:5">
       <c r="B14" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
     </row>
     <row r="15" spans="1:5">
       <c r="B15" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
     </row>
     <row r="16" spans="1:5">
       <c r="B16" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
@@ -2136,63 +2131,58 @@
     </row>
     <row r="18" spans="1:5">
       <c r="B18" s="6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="B19" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="C19" s="13">
-        <f>B20+100</f>
-        <v>0</v>
+        <v>120</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="E19" s="15">
-        <f>B19+100  (use previous row)</f>
-        <v>0</v>
+        <v>122</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="B20" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="D20" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="C20" s="13">
-        <f>D20*1.1</f>
-        <v>0</v>
-      </c>
-      <c r="D20" s="14" t="s">
+      <c r="E20" s="15" t="s">
         <v>127</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="B21" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21" s="13" t="s">
         <v>129</v>
-      </c>
-      <c r="C21" s="13">
-        <f>SUM(D5:D20)</f>
-        <v>0</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="E21" s="15">
-        <f>SUM(D5:D19)  (exclude current row)</f>
-        <v>0</v>
+      <c r="E21" s="15" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2227,7 +2217,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="50" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2237,7 +2227,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2247,7 +2237,7 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -2257,7 +2247,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -2291,7 +2281,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -2301,10 +2291,10 @@
     </row>
     <row r="10" spans="1:6">
       <c r="B10" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -2312,10 +2302,10 @@
     </row>
     <row r="11" spans="1:6">
       <c r="B11" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
@@ -2323,10 +2313,10 @@
     </row>
     <row r="12" spans="1:6">
       <c r="B12" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
@@ -2334,10 +2324,10 @@
     </row>
     <row r="13" spans="1:6">
       <c r="B13" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
@@ -2345,10 +2335,10 @@
     </row>
     <row r="14" spans="1:6">
       <c r="B14" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
@@ -2356,7 +2346,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
@@ -2369,7 +2359,7 @@
         <v>16</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
@@ -2380,7 +2370,7 @@
         <v>18</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
@@ -2391,7 +2381,7 @@
         <v>20</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
@@ -2402,7 +2392,7 @@
         <v>22</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
@@ -2410,10 +2400,10 @@
     </row>
     <row r="20" spans="1:6">
       <c r="B20" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
@@ -2421,7 +2411,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -2431,57 +2421,57 @@
     </row>
     <row r="22" spans="1:6">
       <c r="B22" s="6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F22" s="6"/>
     </row>
     <row r="23" spans="1:6">
       <c r="B23" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="C23" s="14">
-        <f>E3*F3*(1-G3)</f>
-        <v>0</v>
+        <v>158</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>159</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
     </row>
     <row r="24" spans="1:6">
       <c r="B24" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="C24" s="14">
-        <f>H3*0.10</f>
-        <v>0</v>
+        <v>161</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>162</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
     </row>
     <row r="25" spans="1:6">
       <c r="B25" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="C25" s="14">
-        <f>IF(E3&gt;=100,"Yes","No")</f>
-        <v>0</v>
+        <v>164</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>165</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -2503,9 +2493,9 @@
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="E22:F22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D25:F25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>